<commit_message>
Fix Daniel Reiser Infor username and restore Account Review AI CSV files
Issues fixed:
1. Restored 'Booked Sales - Account Review AI.csv' and 'Invoiced Sales - Account Review AI.csv'
   - These files contain complete seller data (not in Sales Pulse Daily files)
   - Were accidentally deleted during folder organization
2. Updated script to check for local CSV files first, fall back to Sales Pulse Daily
3. Added Daniel Reiser Infor username override: 'dreiser' → 'danireis'

Result: Daniel Reiser's report now shows correct GP data
- Q2 2026 Booked: $659,334 (was $0)
- Q2 2026 Invoiced: $20,481 (was $0)
- Q3 2026 Scheduled: $128,670 (was $0)

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sales Operations/Account Review/output/Account Review - Aaron_Mendoza - Q3_2026.xlsx
+++ b/Sales Operations/Account Review/output/Account Review - Aaron_Mendoza - Q3_2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="118">
   <si>
     <t>Report Generated: 07/16/2026</t>
   </si>
@@ -85,7 +85,7 @@
     <t>Alstom</t>
   </si>
   <si>
-    <t>Alstom Transportation Inc.|Alstom Transport Canada Inc|Alstom Transport Canada Inc.</t>
+    <t>Alstom Transport Canada Inc.|Alstom Transportation Inc.|Alstom Transport Canada Inc</t>
   </si>
   <si>
     <t>2024-11-12</t>
@@ -118,7 +118,7 @@
     <t>Eastman Kodak Company</t>
   </si>
   <si>
-    <t>EASTMAN KODAK COMPANY|Kodak Canada ULC</t>
+    <t>Kodak Canada ULC|EASTMAN KODAK COMPANY</t>
   </si>
   <si>
     <t>2024-11-22</t>
@@ -271,7 +271,7 @@
     <t>Advanced Technology Co.</t>
   </si>
   <si>
-    <t>Advanced Manufacturing Corporation Pte. Ltd.|Advanced Technology Co.</t>
+    <t>Advanced Technology Co.|Advanced Manufacturing Corporation Pte. Ltd.</t>
   </si>
   <si>
     <t>Apollo America Inc.</t>
@@ -341,12 +341,6 @@
   </si>
   <si>
     <t>Wincomm International</t>
-  </si>
-  <si>
-    <t>BDI USA</t>
-  </si>
-  <si>
-    <t>GE Medical Systems Information Technologies, Inc</t>
   </si>
   <si>
     <t>NOT ASSIGNED TOTAL</t>
@@ -893,7 +887,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R65"/>
+  <dimension ref="A1:R63"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1133,13 +1127,13 @@
         <v>20186</v>
       </c>
       <c r="M7" s="8">
-        <v>22079.730000000003</v>
+        <v>13047.030000000002</v>
       </c>
       <c r="N7" s="11">
-        <v>0.9142321939625166</v>
+        <v>1.5471720383872802</v>
       </c>
       <c r="O7" s="9">
-        <v>0.4400717756276183</v>
+        <v>0.37200765056053364</v>
       </c>
       <c r="P7" s="8">
         <v>7656</v>
@@ -1342,13 +1336,13 @@
         <v>9701</v>
       </c>
       <c r="M11" s="8">
-        <v>9700.92</v>
+        <v>5244.92</v>
       </c>
       <c r="N11" s="11">
-        <v>1.000008246640525</v>
+        <v>1.849599231256149</v>
       </c>
       <c r="O11" s="9">
-        <v>0.1933493339647484</v>
+        <v>0.14954747299408017</v>
       </c>
       <c r="P11" s="8">
         <v>0</v>
@@ -1446,19 +1440,19 @@
         <v>0.5</v>
       </c>
       <c r="L13" s="8">
-        <v>2771</v>
+        <v>800</v>
       </c>
       <c r="M13" s="8">
         <v>799.96</v>
       </c>
       <c r="N13" s="11">
-        <v>3.463923196159808</v>
+        <v>1.0000500025001249</v>
       </c>
       <c r="O13" s="9">
-        <v>0.0159440272879727</v>
+        <v>0.02280911748822563</v>
       </c>
       <c r="P13" s="8">
-        <v>25500</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="8" t="s">
         <v>1</v>
@@ -1763,16 +1757,16 @@
         <v>5472</v>
       </c>
       <c r="M19" s="8">
-        <v>13441.779999999999</v>
+        <v>13441.78</v>
       </c>
       <c r="N19" s="11">
-        <v>0.40708894208951496</v>
+        <v>0.4070889420895149</v>
       </c>
       <c r="O19" s="9">
-        <v>0.2679085293251233</v>
+        <v>0.38326308724296404</v>
       </c>
       <c r="P19" s="8">
-        <v>7140</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="8" t="s">
         <v>1</v>
@@ -1819,13 +1813,11 @@
         <v>1612</v>
       </c>
       <c r="M20" s="8">
-        <v>1612.38</v>
-      </c>
-      <c r="N20" s="11">
-        <v>0.9997643235465584</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N20" s="5"/>
       <c r="O20" s="9">
-        <v>0.03213639521798768</v>
+        <v>0</v>
       </c>
       <c r="P20" s="8">
         <v>0</v>
@@ -1881,10 +1873,10 @@
         <v>0</v>
       </c>
       <c r="O21" s="9">
-        <v>0.02486196764715379</v>
+        <v>0.03556689478825523</v>
       </c>
       <c r="P21" s="8">
-        <v>1363</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="8" t="s">
         <v>1</v>
@@ -1937,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="9">
-        <v>0.025727970929395917</v>
+        <v>0.03680577692594136</v>
       </c>
       <c r="P22" s="8">
         <v>0</v>
@@ -2188,19 +2180,19 @@
         <v>0.4</v>
       </c>
       <c r="L27" s="15">
-        <v>39742</v>
+        <v>37771</v>
       </c>
       <c r="M27" s="15">
-        <v>50173.02</v>
+        <v>35071.94</v>
       </c>
       <c r="N27" s="16">
-        <v>0.7920990205492913</v>
+        <v>1.0769578187006479</v>
       </c>
       <c r="O27" s="17">
         <v>1</v>
       </c>
       <c r="P27" s="15">
-        <v>41659</v>
+        <v>7656</v>
       </c>
       <c r="Q27" s="12" t="s">
         <v>1</v>
@@ -2361,7 +2353,7 @@
         <v>0</v>
       </c>
       <c r="P31" s="8">
-        <v>2375</v>
+        <v>0</v>
       </c>
       <c r="Q31" s="8" t="s">
         <v>1</v>
@@ -3519,379 +3511,375 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B54" t="s">
+    <row r="54" spans="1:18" s="19" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="C54" s="5">
-        <v>0</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E54" t="s">
-        <v>1</v>
-      </c>
-      <c r="F54" t="s">
-        <v>1</v>
-      </c>
-      <c r="G54" s="5">
-        <v>0</v>
-      </c>
-      <c r="H54" s="5">
-        <v>0</v>
-      </c>
-      <c r="I54" s="5">
-        <v>0</v>
-      </c>
-      <c r="J54" s="5">
-        <v>0</v>
-      </c>
-      <c r="L54" s="8">
-        <v>1538</v>
-      </c>
-      <c r="M54" s="8">
-        <v>0</v>
-      </c>
-      <c r="N54" s="5"/>
-      <c r="O54" s="9">
-        <v>0</v>
-      </c>
-      <c r="P54" s="8">
-        <v>1538</v>
-      </c>
-      <c r="Q54" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="R54" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B55" t="s">
+      <c r="B54" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C54" s="20">
+        <v>139</v>
+      </c>
+      <c r="D54" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="E54" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="F54" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="G54" s="20">
+        <v>104</v>
+      </c>
+      <c r="H54" s="20">
+        <v>44</v>
+      </c>
+      <c r="I54" s="20">
+        <v>21</v>
+      </c>
+      <c r="J54" s="20">
+        <v>6</v>
+      </c>
+      <c r="K54" s="21">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="L54" s="22">
+        <v>4213</v>
+      </c>
+      <c r="M54" s="22">
+        <v>2238</v>
+      </c>
+      <c r="N54" s="23">
+        <v>1.88248436103664</v>
+      </c>
+      <c r="O54" s="24">
+        <v>1</v>
+      </c>
+      <c r="P54" s="22">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="R54" s="19" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="25" t="s">
         <v>111</v>
       </c>
-      <c r="C55" s="5">
-        <v>0</v>
-      </c>
-      <c r="D55" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E55" t="s">
-        <v>1</v>
-      </c>
-      <c r="F55" t="s">
-        <v>1</v>
-      </c>
-      <c r="G55" s="5">
-        <v>0</v>
-      </c>
-      <c r="H55" s="5">
-        <v>0</v>
-      </c>
-      <c r="I55" s="5">
-        <v>0</v>
-      </c>
-      <c r="J55" s="5">
-        <v>0</v>
-      </c>
-      <c r="L55" s="8">
-        <v>0</v>
-      </c>
-      <c r="M55" s="8">
-        <v>0</v>
-      </c>
-      <c r="N55" s="5"/>
-      <c r="O55" s="9">
-        <v>0</v>
-      </c>
-      <c r="P55" s="8">
-        <v>4605</v>
-      </c>
-      <c r="Q55" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="R55" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:18" s="19" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="19" t="s">
+      <c r="B56" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C56" s="26">
+        <v>186</v>
+      </c>
+      <c r="D56" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="E56" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="F56" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="G56" s="26">
+        <v>717</v>
+      </c>
+      <c r="H56" s="26">
+        <v>190</v>
+      </c>
+      <c r="I56" s="26">
+        <v>91</v>
+      </c>
+      <c r="J56" s="26">
+        <v>34</v>
+      </c>
+      <c r="K56" s="27">
+        <v>0.37362637362637363</v>
+      </c>
+      <c r="L56" s="28">
+        <v>41984</v>
+      </c>
+      <c r="M56" s="28">
+        <v>37309.94</v>
+      </c>
+      <c r="N56" s="29">
+        <v>1.1252765348858775</v>
+      </c>
+      <c r="O56" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="P56" s="28">
+        <v>7656</v>
+      </c>
+      <c r="Q56" s="28">
+        <f>SUM(Q6:Q55)</f>
+      </c>
+      <c r="R56" s="25" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="B56" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="C56" s="20">
-        <v>139</v>
-      </c>
-      <c r="D56" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E56" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="F56" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="G56" s="20">
-        <v>104</v>
-      </c>
-      <c r="H56" s="20">
-        <v>44</v>
-      </c>
-      <c r="I56" s="20">
-        <v>21</v>
-      </c>
-      <c r="J56" s="20">
-        <v>6</v>
-      </c>
-      <c r="K56" s="21">
-        <v>0.2857142857142857</v>
-      </c>
-      <c r="L56" s="22">
-        <v>5751</v>
-      </c>
-      <c r="M56" s="22">
-        <v>2238</v>
-      </c>
-      <c r="N56" s="23">
-        <v>2.56970509383378</v>
-      </c>
-      <c r="O56" s="24">
-        <v>1</v>
-      </c>
-      <c r="P56" s="22">
-        <v>8518</v>
-      </c>
-      <c r="Q56" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="R56" s="19" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="25" t="s">
+      <c r="B57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="C57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="D57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="E57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="F57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="G57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="H57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="I57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="J57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="K57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="L57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="M57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="N57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="O57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="P57" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q57" s="31">
+        <v>120000</v>
+      </c>
+      <c r="R57" s="30" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="B58" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="C58" s="26">
-        <v>186</v>
-      </c>
-      <c r="D58" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="E58" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="F58" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="G58" s="26">
-        <v>717</v>
-      </c>
-      <c r="H58" s="26">
-        <v>190</v>
-      </c>
-      <c r="I58" s="26">
-        <v>91</v>
-      </c>
-      <c r="J58" s="26">
-        <v>34</v>
-      </c>
-      <c r="K58" s="27">
-        <v>0.37362637362637363</v>
-      </c>
-      <c r="L58" s="28">
-        <v>45493</v>
-      </c>
-      <c r="M58" s="28">
-        <v>52411.02</v>
-      </c>
-      <c r="N58" s="29">
-        <v>0.8680044769210751</v>
-      </c>
-      <c r="O58" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="P58" s="28">
-        <v>50177</v>
-      </c>
-      <c r="Q58" s="28">
-        <f>SUM(Q6:Q57)</f>
-      </c>
-      <c r="R58" s="25" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:18" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="30" t="s">
+      <c r="B58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="C58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="D58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="E58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="F58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="G58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="H58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="I58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="J58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="K58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="L58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="M58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="N58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="O58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="P58" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q58" s="32">
+        <f>Q56-Q57</f>
+      </c>
+      <c r="R58" s="30" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="B59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="C59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="D59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="E59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="F59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="G59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="H59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="I59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="J59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="K59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="L59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="M59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="N59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="O59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="P59" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q59" s="31">
-        <v>120000</v>
-      </c>
-      <c r="R59" s="30" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:18" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="30" t="s">
+      <c r="B60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="D60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="E60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="F60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="G60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="H60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="I60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="J60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="K60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="L60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="M60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="N60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="O60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="P60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q60" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="R60" s="33" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="34" t="s">
         <v>115</v>
       </c>
-      <c r="B60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="C60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="D60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="E60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="F60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="G60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="H60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="I60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="J60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="K60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="L60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="M60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="N60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="O60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="P60" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q60" s="32">
-        <f>Q58-Q59</f>
-      </c>
-      <c r="R60" s="30" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:18" s="33" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="33" t="s">
+      <c r="B61" s="34"/>
+      <c r="C61" s="34"/>
+      <c r="D61" s="34"/>
+      <c r="E61" s="34"/>
+      <c r="F61" s="34"/>
+      <c r="G61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="H61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="I61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="J61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="K61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="L61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="M61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="N61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="O61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="P61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q61" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="R61" s="34" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="34" t="s">
         <v>116</v>
       </c>
-      <c r="B62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="C62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="D62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="E62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="F62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="G62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="H62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="I62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="J62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="K62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="L62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="M62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="N62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="O62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="P62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q62" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="R62" s="33" t="s">
+      <c r="B62" s="34"/>
+      <c r="C62" s="34"/>
+      <c r="D62" s="34"/>
+      <c r="E62" s="34"/>
+      <c r="F62" s="34"/>
+      <c r="G62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="H62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="I62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="J62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="K62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="L62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="M62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="N62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="O62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="P62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q62" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="R62" s="34" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3941,106 +3929,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:18" s="34" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="34" t="s">
-        <v>118</v>
-      </c>
-      <c r="B64" s="34"/>
-      <c r="C64" s="34"/>
-      <c r="D64" s="34"/>
-      <c r="E64" s="34"/>
-      <c r="F64" s="34"/>
-      <c r="G64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="H64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="I64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="J64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="K64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="L64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="M64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="N64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="O64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="P64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q64" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="R64" s="34" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:18" s="34" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="34" t="s">
-        <v>119</v>
-      </c>
-      <c r="B65" s="34"/>
-      <c r="C65" s="34"/>
-      <c r="D65" s="34"/>
-      <c r="E65" s="34"/>
-      <c r="F65" s="34"/>
-      <c r="G65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="H65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="I65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="J65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="K65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="L65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="M65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="N65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="O65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="P65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q65" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="R65" s="34" t="s">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A61:F61"/>
+    <mergeCell ref="A62:F62"/>
     <mergeCell ref="A63:F63"/>
-    <mergeCell ref="A64:F64"/>
-    <mergeCell ref="A65:F65"/>
   </mergeCells>
-  <conditionalFormatting sqref="Q60">
+  <conditionalFormatting sqref="Q58">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>